<commit_message>
Voucher Details Adjustments WIP
</commit_message>
<xml_diff>
--- a/Template/Voucher Template - 2.xlsx
+++ b/Template/Voucher Template - 2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Smart Travel PC\Desktop\Vouchers Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C460458-F3A5-40F0-B618-B471513112C4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48C9C5BF-CF53-4C93-A6C3-FB61AF45AA22}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="675" windowWidth="19935" windowHeight="15525" xr2:uid="{46FCF62E-0F38-40EF-B40B-6239A54C7BFA}"/>
+    <workbookView xWindow="1170" yWindow="675" windowWidth="19935" windowHeight="15525" xr2:uid="{46FCF62E-0F38-40EF-B40B-6239A54C7BFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
   <si>
     <t>TO:</t>
   </si>
@@ -169,6 +169,21 @@
   </si>
   <si>
     <t>*** It will be subject to change based on the local situation ***</t>
+  </si>
+  <si>
+    <t>To</t>
+  </si>
+  <si>
+    <t>2N</t>
+  </si>
+  <si>
+    <t>SEOUL</t>
+  </si>
+  <si>
+    <t>SMART STAY HOTEL</t>
+  </si>
+  <si>
+    <t>686F25BBF011A</t>
   </si>
 </sst>
 </file>
@@ -440,7 +455,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -554,18 +569,21 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -575,38 +593,71 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -697,6 +748,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -719,23 +776,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>19049</xdr:rowOff>
+      <xdr:rowOff>85725</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>876300</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>723900</xdr:rowOff>
+      <xdr:rowOff>685800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D0BDFC6A-3B55-4B5E-ABF3-1BFC47E49B9C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1473BF12-162B-4568-9D6D-BA45B3FCFE42}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -743,21 +800,22 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect l="14562" t="38950" r="24164" b="43105"/>
-        <a:stretch/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1752600" y="19049"/>
-          <a:ext cx="2924175" cy="704851"/>
+          <a:off x="9525" y="85725"/>
+          <a:ext cx="6657975" cy="600075"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1095,37 +1153,39 @@
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="78" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="70"/>
+      <c r="B2" s="79"/>
+      <c r="C2" s="80" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="81"/>
+      <c r="E2" s="82"/>
       <c r="F2" s="13"/>
       <c r="G2" s="14"/>
       <c r="H2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="20"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="19"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="70"/>
       <c r="N2" s="2"/>
     </row>
     <row r="3" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
-      <c r="G3" s="59"/>
-      <c r="H3" s="59"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="60"/>
+      <c r="B3" s="71"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="72"/>
       <c r="N3" s="2"/>
     </row>
     <row r="4" spans="1:14" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1146,63 +1206,63 @@
       <c r="A5" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="74" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="62"/>
-      <c r="D5" s="62"/>
-      <c r="E5" s="62"/>
-      <c r="F5" s="64" t="s">
+      <c r="C5" s="74"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="76" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="65"/>
+      <c r="G5" s="77"/>
       <c r="H5" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="61"/>
-      <c r="J5" s="61"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="73"/>
       <c r="K5" s="19"/>
     </row>
     <row r="6" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="74" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="64" t="s">
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="65"/>
+      <c r="G6" s="77"/>
       <c r="H6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="61"/>
-      <c r="J6" s="61"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="73"/>
       <c r="K6" s="19"/>
     </row>
     <row r="7" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="63" t="s">
+      <c r="B7" s="75" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="63"/>
-      <c r="D7" s="63"/>
-      <c r="E7" s="63"/>
-      <c r="F7" s="64" t="s">
+      <c r="C7" s="75"/>
+      <c r="D7" s="75"/>
+      <c r="E7" s="75"/>
+      <c r="F7" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="65"/>
+      <c r="G7" s="77"/>
       <c r="H7" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61"/>
+      <c r="I7" s="73"/>
+      <c r="J7" s="73"/>
       <c r="K7" s="19"/>
     </row>
     <row r="8" spans="1:14" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1249,10 +1309,10 @@
     <row r="11" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="35"/>
       <c r="B11" s="36"/>
-      <c r="C11" s="43" t="s">
+      <c r="C11" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="44"/>
+      <c r="D11" s="42"/>
       <c r="E11" s="8" t="s">
         <v>16</v>
       </c>
@@ -1260,60 +1320,70 @@
         <v>17</v>
       </c>
       <c r="G11" s="57"/>
-      <c r="H11" s="43" t="s">
+      <c r="H11" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="I11" s="58"/>
-      <c r="J11" s="58"/>
-      <c r="K11" s="44"/>
+      <c r="I11" s="67"/>
+      <c r="J11" s="67"/>
+      <c r="K11" s="42"/>
     </row>
     <row r="12" spans="1:14" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="37"/>
       <c r="B12" s="38"/>
-      <c r="C12" s="48"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
-      <c r="K12" s="28"/>
+      <c r="C12" s="51">
+        <v>45855</v>
+      </c>
+      <c r="D12" s="52"/>
+      <c r="E12" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="58" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" s="60"/>
+      <c r="H12" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="I12" s="59"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="60"/>
     </row>
     <row r="13" spans="1:14" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="39"/>
       <c r="B13" s="40"/>
-      <c r="C13" s="50"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="46"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="29"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
-      <c r="K13" s="31"/>
-    </row>
-    <row r="14" spans="1:14" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C13" s="53"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="63"/>
+      <c r="H13" s="61"/>
+      <c r="I13" s="62"/>
+      <c r="J13" s="62"/>
+      <c r="K13" s="63"/>
+    </row>
+    <row r="14" spans="1:14" s="4" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="39"/>
       <c r="B14" s="40"/>
-      <c r="C14" s="50"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="32"/>
-      <c r="I14" s="33"/>
-      <c r="J14" s="33"/>
-      <c r="K14" s="34"/>
-    </row>
-    <row r="15" spans="1:14" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C14" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="50"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="64"/>
+      <c r="I14" s="65"/>
+      <c r="J14" s="65"/>
+      <c r="K14" s="66"/>
+    </row>
+    <row r="15" spans="1:14" s="4" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="39"/>
       <c r="B15" s="40"/>
-      <c r="C15" s="52"/>
-      <c r="D15" s="53"/>
-      <c r="E15" s="46"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="31"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="63"/>
       <c r="H15" s="26"/>
       <c r="I15" s="27"/>
       <c r="J15" s="27"/>
@@ -1322,11 +1392,13 @@
     <row r="16" spans="1:14" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="39"/>
       <c r="B16" s="40"/>
-      <c r="C16" s="54"/>
-      <c r="D16" s="53"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="31"/>
+      <c r="C16" s="53">
+        <v>45855</v>
+      </c>
+      <c r="D16" s="54"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="61"/>
+      <c r="G16" s="63"/>
       <c r="H16" s="29"/>
       <c r="I16" s="30"/>
       <c r="J16" s="30"/>
@@ -1337,9 +1409,9 @@
       <c r="B17" s="40"/>
       <c r="C17" s="55"/>
       <c r="D17" s="56"/>
-      <c r="E17" s="47"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="34"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="64"/>
+      <c r="G17" s="66"/>
       <c r="H17" s="32"/>
       <c r="I17" s="33"/>
       <c r="J17" s="33"/>
@@ -1348,9 +1420,9 @@
     <row r="18" spans="1:11" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="39"/>
       <c r="B18" s="40"/>
-      <c r="C18" s="48"/>
-      <c r="D18" s="49"/>
-      <c r="E18" s="45"/>
+      <c r="C18" s="51"/>
+      <c r="D18" s="52"/>
+      <c r="E18" s="46"/>
       <c r="F18" s="26"/>
       <c r="G18" s="28"/>
       <c r="H18" s="26"/>
@@ -1361,9 +1433,9 @@
     <row r="19" spans="1:11" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="39"/>
       <c r="B19" s="40"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="46"/>
+      <c r="C19" s="53"/>
+      <c r="D19" s="54"/>
+      <c r="E19" s="47"/>
       <c r="F19" s="29"/>
       <c r="G19" s="31"/>
       <c r="H19" s="29"/>
@@ -1371,12 +1443,14 @@
       <c r="J19" s="30"/>
       <c r="K19" s="31"/>
     </row>
-    <row r="20" spans="1:11" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:11" s="4" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="39"/>
       <c r="B20" s="40"/>
-      <c r="C20" s="50"/>
-      <c r="D20" s="51"/>
-      <c r="E20" s="46"/>
+      <c r="C20" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="50"/>
+      <c r="E20" s="47"/>
       <c r="F20" s="29"/>
       <c r="G20" s="31"/>
       <c r="H20" s="32"/>
@@ -1384,12 +1458,12 @@
       <c r="J20" s="33"/>
       <c r="K20" s="34"/>
     </row>
-    <row r="21" spans="1:11" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:11" s="4" customFormat="1" ht="8.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="39"/>
       <c r="B21" s="40"/>
-      <c r="C21" s="52"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="46"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="47"/>
       <c r="F21" s="29"/>
       <c r="G21" s="31"/>
       <c r="H21" s="26"/>
@@ -1400,9 +1474,9 @@
     <row r="22" spans="1:11" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="39"/>
       <c r="B22" s="40"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="53"/>
-      <c r="E22" s="46"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="47"/>
       <c r="F22" s="29"/>
       <c r="G22" s="31"/>
       <c r="H22" s="29"/>
@@ -1411,11 +1485,11 @@
       <c r="K22" s="31"/>
     </row>
     <row r="23" spans="1:11" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="41"/>
-      <c r="B23" s="42"/>
-      <c r="C23" s="55"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="47"/>
+      <c r="A23" s="39"/>
+      <c r="B23" s="40"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="102"/>
+      <c r="E23" s="48"/>
       <c r="F23" s="32"/>
       <c r="G23" s="34"/>
       <c r="H23" s="32"/>
@@ -1428,39 +1502,39 @@
       <c r="A25" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B25" s="76"/>
-      <c r="C25" s="77" t="s">
+      <c r="B25" s="88"/>
+      <c r="C25" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="77"/>
-      <c r="F25" s="77"/>
-      <c r="G25" s="77"/>
-      <c r="H25" s="77"/>
-      <c r="I25" s="77"/>
-      <c r="J25" s="77"/>
-      <c r="K25" s="77"/>
+      <c r="D25" s="89"/>
+      <c r="E25" s="89"/>
+      <c r="F25" s="89"/>
+      <c r="G25" s="89"/>
+      <c r="H25" s="89"/>
+      <c r="I25" s="89"/>
+      <c r="J25" s="89"/>
+      <c r="K25" s="89"/>
     </row>
     <row r="26" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="76"/>
-      <c r="B26" s="76"/>
-      <c r="C26" s="77"/>
-      <c r="D26" s="77"/>
-      <c r="E26" s="77"/>
-      <c r="F26" s="77"/>
-      <c r="G26" s="77"/>
-      <c r="H26" s="77"/>
-      <c r="I26" s="77"/>
-      <c r="J26" s="77"/>
-      <c r="K26" s="77"/>
+      <c r="A26" s="88"/>
+      <c r="B26" s="88"/>
+      <c r="C26" s="89"/>
+      <c r="D26" s="89"/>
+      <c r="E26" s="89"/>
+      <c r="F26" s="89"/>
+      <c r="G26" s="89"/>
+      <c r="H26" s="89"/>
+      <c r="I26" s="89"/>
+      <c r="J26" s="89"/>
+      <c r="K26" s="89"/>
     </row>
     <row r="27" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="81" t="s">
+      <c r="A27" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="B27" s="82"/>
-      <c r="C27" s="76"/>
-      <c r="D27" s="76"/>
+      <c r="B27" s="94"/>
+      <c r="C27" s="88"/>
+      <c r="D27" s="88"/>
       <c r="E27" s="7" t="s">
         <v>4</v>
       </c>
@@ -1478,12 +1552,12 @@
       <c r="K27" s="24"/>
     </row>
     <row r="28" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="83"/>
-      <c r="B28" s="84"/>
-      <c r="C28" s="87" t="s">
+      <c r="A28" s="95"/>
+      <c r="B28" s="96"/>
+      <c r="C28" s="99" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="88"/>
+      <c r="D28" s="100"/>
       <c r="E28" s="11" t="s">
         <v>30</v>
       </c>
@@ -1501,12 +1575,12 @@
       <c r="K28" s="22"/>
     </row>
     <row r="29" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="85"/>
-      <c r="B29" s="86"/>
-      <c r="C29" s="87" t="s">
+      <c r="A29" s="97"/>
+      <c r="B29" s="98"/>
+      <c r="C29" s="99" t="s">
         <v>21</v>
       </c>
-      <c r="D29" s="88"/>
+      <c r="D29" s="100"/>
       <c r="E29" s="11" t="s">
         <v>31</v>
       </c>
@@ -1527,7 +1601,7 @@
       <c r="A30" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="76"/>
+      <c r="B30" s="88"/>
       <c r="C30" s="24" t="s">
         <v>4</v>
       </c>
@@ -1545,8 +1619,8 @@
       <c r="K30" s="24"/>
     </row>
     <row r="31" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="76"/>
-      <c r="B31" s="76"/>
+      <c r="A31" s="88"/>
+      <c r="B31" s="88"/>
       <c r="C31" s="22" t="s">
         <v>36</v>
       </c>
@@ -1564,8 +1638,8 @@
       <c r="K31" s="22"/>
     </row>
     <row r="32" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="76"/>
-      <c r="B32" s="76"/>
+      <c r="A32" s="88"/>
+      <c r="B32" s="88"/>
       <c r="C32" s="22"/>
       <c r="D32" s="22"/>
       <c r="E32" s="23"/>
@@ -1654,74 +1728,74 @@
     <row r="38" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="24"/>
       <c r="B38" s="24"/>
-      <c r="C38" s="71"/>
-      <c r="D38" s="72"/>
-      <c r="E38" s="72"/>
-      <c r="F38" s="72"/>
-      <c r="G38" s="72"/>
-      <c r="H38" s="72"/>
-      <c r="I38" s="72"/>
-      <c r="J38" s="72"/>
-      <c r="K38" s="73"/>
+      <c r="C38" s="83"/>
+      <c r="D38" s="84"/>
+      <c r="E38" s="84"/>
+      <c r="F38" s="84"/>
+      <c r="G38" s="84"/>
+      <c r="H38" s="84"/>
+      <c r="I38" s="84"/>
+      <c r="J38" s="84"/>
+      <c r="K38" s="85"/>
     </row>
     <row r="39" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
-      <c r="C39" s="71"/>
-      <c r="D39" s="72"/>
-      <c r="E39" s="72"/>
-      <c r="F39" s="72"/>
-      <c r="G39" s="72"/>
-      <c r="H39" s="72"/>
-      <c r="I39" s="72"/>
-      <c r="J39" s="72"/>
-      <c r="K39" s="73"/>
+      <c r="C39" s="83"/>
+      <c r="D39" s="84"/>
+      <c r="E39" s="84"/>
+      <c r="F39" s="84"/>
+      <c r="G39" s="84"/>
+      <c r="H39" s="84"/>
+      <c r="I39" s="84"/>
+      <c r="J39" s="84"/>
+      <c r="K39" s="85"/>
     </row>
     <row r="40" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="24"/>
       <c r="B40" s="24"/>
-      <c r="C40" s="78"/>
-      <c r="D40" s="79"/>
-      <c r="E40" s="79"/>
-      <c r="F40" s="79"/>
-      <c r="G40" s="79"/>
-      <c r="H40" s="79"/>
-      <c r="I40" s="79"/>
-      <c r="J40" s="79"/>
-      <c r="K40" s="80"/>
+      <c r="C40" s="90"/>
+      <c r="D40" s="91"/>
+      <c r="E40" s="91"/>
+      <c r="F40" s="91"/>
+      <c r="G40" s="91"/>
+      <c r="H40" s="91"/>
+      <c r="I40" s="91"/>
+      <c r="J40" s="91"/>
+      <c r="K40" s="92"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="24" t="s">
         <v>26</v>
       </c>
       <c r="B41" s="24"/>
-      <c r="C41" s="74" t="s">
+      <c r="C41" s="86" t="s">
         <v>47</v>
       </c>
-      <c r="D41" s="75"/>
-      <c r="E41" s="75"/>
-      <c r="F41" s="75"/>
-      <c r="G41" s="75"/>
-      <c r="H41" s="75"/>
-      <c r="I41" s="75"/>
-      <c r="J41" s="75"/>
-      <c r="K41" s="75"/>
+      <c r="D41" s="87"/>
+      <c r="E41" s="87"/>
+      <c r="F41" s="87"/>
+      <c r="G41" s="87"/>
+      <c r="H41" s="87"/>
+      <c r="I41" s="87"/>
+      <c r="J41" s="87"/>
+      <c r="K41" s="87"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="24"/>
       <c r="B42" s="24"/>
-      <c r="C42" s="75"/>
-      <c r="D42" s="75"/>
-      <c r="E42" s="75"/>
-      <c r="F42" s="75"/>
-      <c r="G42" s="75"/>
-      <c r="H42" s="75"/>
-      <c r="I42" s="75"/>
-      <c r="J42" s="75"/>
-      <c r="K42" s="75"/>
+      <c r="C42" s="87"/>
+      <c r="D42" s="87"/>
+      <c r="E42" s="87"/>
+      <c r="F42" s="87"/>
+      <c r="G42" s="87"/>
+      <c r="H42" s="87"/>
+      <c r="I42" s="87"/>
+      <c r="J42" s="87"/>
+      <c r="K42" s="87"/>
     </row>
   </sheetData>
-  <mergeCells count="65">
+  <mergeCells count="67">
     <mergeCell ref="C39:K39"/>
     <mergeCell ref="A41:B42"/>
     <mergeCell ref="C41:K42"/>
@@ -1765,10 +1839,12 @@
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="E12:E17"/>
     <mergeCell ref="E18:E23"/>
-    <mergeCell ref="C12:D14"/>
-    <mergeCell ref="C15:D17"/>
-    <mergeCell ref="C18:D20"/>
-    <mergeCell ref="C21:D23"/>
+    <mergeCell ref="C14:D15"/>
+    <mergeCell ref="C12:D13"/>
+    <mergeCell ref="C16:D17"/>
+    <mergeCell ref="C20:D21"/>
+    <mergeCell ref="C18:D19"/>
+    <mergeCell ref="C22:D23"/>
     <mergeCell ref="A33:B36"/>
     <mergeCell ref="C33:K33"/>
     <mergeCell ref="C34:K34"/>

</xml_diff>